<commit_message>
Make project work with real HHs data on ResearchCloud
</commit_message>
<xml_diff>
--- a/R/data/df_persona_per_group.xlsx
+++ b/R/data/df_persona_per_group.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AE15"/>
+  <dimension ref="A1:AE18"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -523,13 +523,13 @@
         </is>
       </c>
       <c r="C2">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D2">
-        <v>915</v>
+        <v>1078</v>
       </c>
       <c r="E2">
-        <v>0.5669999999999999</v>
+        <v>0.482</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
@@ -558,7 +558,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -595,31 +595,31 @@
         <v>20</v>
       </c>
       <c r="S2">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="T2">
-        <v>32.4</v>
+        <v>34.3</v>
       </c>
       <c r="U2">
+        <v>6.5</v>
+      </c>
+      <c r="V2">
+        <v>6.5</v>
+      </c>
+      <c r="W2">
+        <v>6.1</v>
+      </c>
+      <c r="X2">
         <v>6.4</v>
       </c>
-      <c r="V2">
-        <v>6.4</v>
-      </c>
-      <c r="W2">
-        <v>5.9</v>
-      </c>
-      <c r="X2">
-        <v>6.3</v>
-      </c>
       <c r="Y2">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z2">
         <v>6.2</v>
       </c>
       <c r="AA2">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AB2">
         <v>0</v>
@@ -628,7 +628,7 @@
         <v>0</v>
       </c>
       <c r="AD2">
-        <v>2016</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="3">
@@ -643,13 +643,13 @@
         </is>
       </c>
       <c r="C3">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D3">
-        <v>698</v>
+        <v>1159</v>
       </c>
       <c r="E3">
-        <v>0.433</v>
+        <v>0.518</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -663,12 +663,12 @@
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>HAVO</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>EM&amp;CM</t>
+          <t>EM</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -678,12 +678,12 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="M3" t="inlineStr">
@@ -715,31 +715,31 @@
         <v>19</v>
       </c>
       <c r="S3">
-        <v>137</v>
+        <v>147</v>
       </c>
       <c r="T3">
-        <v>33.4</v>
+        <v>34.3</v>
       </c>
       <c r="U3">
+        <v>6.5</v>
+      </c>
+      <c r="V3">
+        <v>6.5</v>
+      </c>
+      <c r="W3">
+        <v>6.1</v>
+      </c>
+      <c r="X3">
         <v>6.4</v>
       </c>
-      <c r="V3">
-        <v>6.4</v>
-      </c>
-      <c r="W3">
-        <v>5.9</v>
-      </c>
-      <c r="X3">
-        <v>6.3</v>
-      </c>
       <c r="Y3">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z3">
         <v>6.2</v>
       </c>
       <c r="AA3">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AB3">
         <v>0</v>
@@ -748,7 +748,7 @@
         <v>0</v>
       </c>
       <c r="AD3">
-        <v>2017</v>
+        <v>2021</v>
       </c>
     </row>
     <row r="4">
@@ -763,17 +763,17 @@
         </is>
       </c>
       <c r="C4">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D4">
-        <v>756</v>
+        <v>755</v>
       </c>
       <c r="E4">
-        <v>0.469</v>
+        <v>0.338</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>V</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
@@ -788,7 +788,7 @@
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>MedV</t>
+          <t>EM</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -835,31 +835,31 @@
         <v>19</v>
       </c>
       <c r="S4">
-        <v>137.5</v>
+        <v>154</v>
       </c>
       <c r="T4">
-        <v>34.2</v>
+        <v>34.3</v>
       </c>
       <c r="U4">
+        <v>6.5</v>
+      </c>
+      <c r="V4">
+        <v>6.5</v>
+      </c>
+      <c r="W4">
+        <v>6.1</v>
+      </c>
+      <c r="X4">
         <v>6.4</v>
       </c>
-      <c r="V4">
-        <v>6.4</v>
-      </c>
-      <c r="W4">
-        <v>5.9</v>
-      </c>
-      <c r="X4">
-        <v>6.3</v>
-      </c>
       <c r="Y4">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z4">
         <v>6.2</v>
       </c>
       <c r="AA4">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AB4">
         <v>0</v>
@@ -868,7 +868,7 @@
         <v>0</v>
       </c>
       <c r="AD4">
-        <v>2016</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="5">
@@ -883,13 +883,13 @@
         </is>
       </c>
       <c r="C5">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D5">
-        <v>176</v>
+        <v>311</v>
       </c>
       <c r="E5">
-        <v>0.109</v>
+        <v>0.139</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -903,17 +903,17 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>HAVO</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>MedV</t>
+          <t>EM</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -952,34 +952,34 @@
         </is>
       </c>
       <c r="R5">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S5">
-        <v>134.5</v>
+        <v>162</v>
       </c>
       <c r="T5">
-        <v>34.7</v>
+        <v>34.3</v>
       </c>
       <c r="U5">
+        <v>6.5</v>
+      </c>
+      <c r="V5">
+        <v>6.5</v>
+      </c>
+      <c r="W5">
+        <v>6.1</v>
+      </c>
+      <c r="X5">
         <v>6.4</v>
       </c>
-      <c r="V5">
-        <v>6.4</v>
-      </c>
-      <c r="W5">
-        <v>5.9</v>
-      </c>
-      <c r="X5">
-        <v>6.3</v>
-      </c>
       <c r="Y5">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z5">
         <v>6.2</v>
       </c>
       <c r="AA5">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AB5">
         <v>0</v>
@@ -988,7 +988,7 @@
         <v>0</v>
       </c>
       <c r="AD5">
-        <v>2017</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="6">
@@ -1003,13 +1003,13 @@
         </is>
       </c>
       <c r="C6">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D6">
-        <v>202</v>
+        <v>242</v>
       </c>
       <c r="E6">
-        <v>0.125</v>
+        <v>0.108</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
@@ -1028,7 +1028,7 @@
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>EM&amp;CM</t>
+          <t>EM</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -1038,22 +1038,22 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="M6" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="N6" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
@@ -1075,25 +1075,25 @@
         <v>21</v>
       </c>
       <c r="S6">
-        <v>128.5</v>
+        <v>124</v>
       </c>
       <c r="T6">
-        <v>28.1</v>
+        <v>27.8</v>
       </c>
       <c r="U6">
+        <v>6.5</v>
+      </c>
+      <c r="V6">
+        <v>6.5</v>
+      </c>
+      <c r="W6">
+        <v>6.1</v>
+      </c>
+      <c r="X6">
         <v>6.4</v>
       </c>
-      <c r="V6">
-        <v>6.4</v>
-      </c>
-      <c r="W6">
-        <v>5.9</v>
-      </c>
-      <c r="X6">
-        <v>6.3</v>
-      </c>
       <c r="Y6">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z6">
         <v>6.2</v>
@@ -1108,7 +1108,7 @@
         <v>0</v>
       </c>
       <c r="AD6">
-        <v>2018</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="7">
@@ -1123,13 +1123,13 @@
         </is>
       </c>
       <c r="C7">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D7">
-        <v>445</v>
+        <v>411</v>
       </c>
       <c r="E7">
-        <v>0.276</v>
+        <v>0.184</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="L7" t="inlineStr">
@@ -1168,17 +1168,17 @@
       </c>
       <c r="M7" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="N7" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="P7" t="inlineStr">
@@ -1192,28 +1192,28 @@
         </is>
       </c>
       <c r="R7">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="S7">
-        <v>112</v>
+        <v>126</v>
       </c>
       <c r="T7">
-        <v>36.1</v>
+        <v>34.2</v>
       </c>
       <c r="U7">
+        <v>6.5</v>
+      </c>
+      <c r="V7">
+        <v>6.5</v>
+      </c>
+      <c r="W7">
+        <v>6.1</v>
+      </c>
+      <c r="X7">
         <v>6.4</v>
       </c>
-      <c r="V7">
-        <v>6.4</v>
-      </c>
-      <c r="W7">
-        <v>5.9</v>
-      </c>
-      <c r="X7">
-        <v>6.3</v>
-      </c>
       <c r="Y7">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z7">
         <v>6.2</v>
@@ -1228,7 +1228,7 @@
         <v>0</v>
       </c>
       <c r="AD7">
-        <v>2015</v>
+        <v>2018</v>
       </c>
     </row>
     <row r="8">
@@ -1243,17 +1243,17 @@
         </is>
       </c>
       <c r="C8">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D8">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="E8">
-        <v>0.008999999999999999</v>
+        <v>0.012</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>V</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -1273,7 +1273,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
@@ -1312,28 +1312,28 @@
         </is>
       </c>
       <c r="R8">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="S8">
-        <v>60</v>
+        <v>135</v>
       </c>
       <c r="T8">
-        <v>29.8</v>
+        <v>26.8</v>
       </c>
       <c r="U8">
+        <v>6.5</v>
+      </c>
+      <c r="V8">
+        <v>6.5</v>
+      </c>
+      <c r="W8">
+        <v>6.1</v>
+      </c>
+      <c r="X8">
         <v>6.4</v>
       </c>
-      <c r="V8">
-        <v>6.4</v>
-      </c>
-      <c r="W8">
-        <v>5.9</v>
-      </c>
-      <c r="X8">
-        <v>6.3</v>
-      </c>
       <c r="Y8">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z8">
         <v>6.2</v>
@@ -1342,13 +1342,13 @@
         <v>0</v>
       </c>
       <c r="AB8">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="AC8">
         <v>0</v>
       </c>
       <c r="AD8">
-        <v>2019</v>
+        <v>2022</v>
       </c>
     </row>
     <row r="9">
@@ -1363,13 +1363,13 @@
         </is>
       </c>
       <c r="C9">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D9">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E9">
-        <v>0.012</v>
+        <v>0.008</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1388,12 +1388,12 @@
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>EM&amp;CM</t>
+          <t>EM</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -1435,25 +1435,25 @@
         <v>22</v>
       </c>
       <c r="S9">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="T9">
-        <v>30.5</v>
+        <v>29.7</v>
       </c>
       <c r="U9">
+        <v>6.5</v>
+      </c>
+      <c r="V9">
+        <v>6.5</v>
+      </c>
+      <c r="W9">
+        <v>6.1</v>
+      </c>
+      <c r="X9">
         <v>6.4</v>
       </c>
-      <c r="V9">
-        <v>6.4</v>
-      </c>
-      <c r="W9">
-        <v>5.9</v>
-      </c>
-      <c r="X9">
-        <v>6.3</v>
-      </c>
       <c r="Y9">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z9">
         <v>6.2</v>
@@ -1468,52 +1468,52 @@
         <v>0</v>
       </c>
       <c r="AD9">
-        <v>2012</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Vooropleiding</t>
+          <t>Aansluiting</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>Overig</t>
         </is>
       </c>
       <c r="C10">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D10">
-        <v>522</v>
+        <v>197</v>
       </c>
       <c r="E10">
-        <v>0.324</v>
+        <v>0.08799999999999999</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>V</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Overig</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>MBO</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>MedV</t>
+          <t>EM</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
@@ -1555,25 +1555,25 @@
         <v>21</v>
       </c>
       <c r="S10">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="T10">
-        <v>32.7</v>
+        <v>34.3</v>
       </c>
       <c r="U10">
+        <v>6.5</v>
+      </c>
+      <c r="V10">
+        <v>6.5</v>
+      </c>
+      <c r="W10">
+        <v>6.1</v>
+      </c>
+      <c r="X10">
         <v>6.4</v>
       </c>
-      <c r="V10">
-        <v>6.4</v>
-      </c>
-      <c r="W10">
-        <v>5.9</v>
-      </c>
-      <c r="X10">
-        <v>6.3</v>
-      </c>
       <c r="Y10">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z10">
         <v>6.2</v>
@@ -1588,77 +1588,77 @@
         <v>0</v>
       </c>
       <c r="AD10">
-        <v>2017</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Vooropleiding</t>
+          <t>Aansluiting</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>HAVO</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="C11">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D11">
-        <v>860</v>
+        <v>276</v>
       </c>
       <c r="E11">
-        <v>0.533</v>
+        <v>0.123</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>V</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Direct</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>HAVO</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>EM&amp;CM</t>
+          <t>EM</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="N11" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="P11" t="inlineStr">
@@ -1675,31 +1675,31 @@
         <v>19</v>
       </c>
       <c r="S11">
-        <v>132</v>
+        <v>152</v>
       </c>
       <c r="T11">
-        <v>35.9</v>
+        <v>34.3</v>
       </c>
       <c r="U11">
+        <v>6.5</v>
+      </c>
+      <c r="V11">
+        <v>6.5</v>
+      </c>
+      <c r="W11">
+        <v>6.1</v>
+      </c>
+      <c r="X11">
         <v>6.4</v>
       </c>
-      <c r="V11">
-        <v>6.4</v>
-      </c>
-      <c r="W11">
-        <v>5.9</v>
-      </c>
-      <c r="X11">
-        <v>6.3</v>
-      </c>
       <c r="Y11">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z11">
         <v>6.2</v>
       </c>
       <c r="AA11">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AB11">
         <v>0</v>
@@ -1708,7 +1708,7 @@
         <v>0</v>
       </c>
       <c r="AD11">
-        <v>2016</v>
+        <v>2024</v>
       </c>
     </row>
     <row r="12">
@@ -1719,17 +1719,17 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>VWO</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="C12">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D12">
-        <v>58</v>
+        <v>534</v>
       </c>
       <c r="E12">
-        <v>0.036</v>
+        <v>0.239</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
@@ -1738,12 +1738,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Switch extern</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>VWO</t>
+          <t>MBO</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -1758,27 +1758,27 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="M12" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="N12" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="P12" t="inlineStr">
@@ -1792,34 +1792,34 @@
         </is>
       </c>
       <c r="R12">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="S12">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="T12">
-        <v>30.9</v>
+        <v>32.7</v>
       </c>
       <c r="U12">
+        <v>6.5</v>
+      </c>
+      <c r="V12">
+        <v>6.5</v>
+      </c>
+      <c r="W12">
+        <v>6.1</v>
+      </c>
+      <c r="X12">
         <v>6.4</v>
       </c>
-      <c r="V12">
-        <v>6.4</v>
-      </c>
-      <c r="W12">
-        <v>5.9</v>
-      </c>
-      <c r="X12">
-        <v>6.3</v>
-      </c>
       <c r="Y12">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z12">
         <v>6.2</v>
       </c>
       <c r="AA12">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="AB12">
         <v>0</v>
@@ -1828,7 +1828,7 @@
         <v>0</v>
       </c>
       <c r="AD12">
-        <v>2016</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="13">
@@ -1839,17 +1839,17 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>HAVO</t>
         </is>
       </c>
       <c r="C13">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D13">
-        <v>92</v>
+        <v>733</v>
       </c>
       <c r="E13">
-        <v>0.057</v>
+        <v>0.328</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
@@ -1863,7 +1863,7 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>BD</t>
+          <t>HAVO</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -1873,32 +1873,32 @@
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>Onbekend</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="M13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="N13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="P13" t="inlineStr">
@@ -1912,43 +1912,43 @@
         </is>
       </c>
       <c r="R13">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="S13">
-        <v>126</v>
+        <v>138</v>
       </c>
       <c r="T13">
-        <v>15.5</v>
+        <v>34.3</v>
       </c>
       <c r="U13">
+        <v>6.5</v>
+      </c>
+      <c r="V13">
+        <v>6.5</v>
+      </c>
+      <c r="W13">
+        <v>6.1</v>
+      </c>
+      <c r="X13">
         <v>6.4</v>
       </c>
-      <c r="V13">
-        <v>6.4</v>
-      </c>
-      <c r="W13">
-        <v>5.9</v>
-      </c>
-      <c r="X13">
-        <v>6.3</v>
-      </c>
       <c r="Y13">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z13">
         <v>6.2</v>
       </c>
       <c r="AA13">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB13">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AC13">
         <v>0</v>
       </c>
       <c r="AD13">
-        <v>2017</v>
+        <v>2019</v>
       </c>
     </row>
     <row r="14">
@@ -1959,17 +1959,17 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>VWO</t>
         </is>
       </c>
       <c r="C14">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D14">
-        <v>30</v>
+        <v>115</v>
       </c>
       <c r="E14">
-        <v>0.019</v>
+        <v>0.051</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
@@ -1978,17 +1978,17 @@
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Na CD</t>
+          <t>Switch extern</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>CD</t>
+          <t>VWO</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>EM</t>
+          <t>NT</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1998,27 +1998,27 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="M14" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="N14" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>Ja</t>
+          <t>Nee</t>
         </is>
       </c>
       <c r="P14" t="inlineStr">
@@ -2032,43 +2032,43 @@
         </is>
       </c>
       <c r="R14">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="S14">
-        <v>127.5</v>
+        <v>133</v>
       </c>
       <c r="T14">
-        <v>29.6</v>
+        <v>34.3</v>
       </c>
       <c r="U14">
+        <v>6.5</v>
+      </c>
+      <c r="V14">
+        <v>6.5</v>
+      </c>
+      <c r="W14">
+        <v>6.1</v>
+      </c>
+      <c r="X14">
         <v>6.4</v>
       </c>
-      <c r="V14">
-        <v>6.4</v>
-      </c>
-      <c r="W14">
-        <v>5.9</v>
-      </c>
-      <c r="X14">
-        <v>6.3</v>
-      </c>
       <c r="Y14">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z14">
         <v>6.2</v>
       </c>
       <c r="AA14">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="AB14">
-        <v>-0</v>
+        <v>0.1</v>
       </c>
       <c r="AC14">
         <v>0</v>
       </c>
       <c r="AD14">
-        <v>2017.5</v>
+        <v>2020</v>
       </c>
     </row>
     <row r="15">
@@ -2079,17 +2079,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>HO</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="C15">
-        <v>1613</v>
+        <v>2237</v>
       </c>
       <c r="D15">
-        <v>51</v>
+        <v>749</v>
       </c>
       <c r="E15">
-        <v>0.032</v>
+        <v>0.335</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
@@ -2098,12 +2098,12 @@
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Switch extern</t>
+          <t>Direct</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>HO</t>
+          <t>BD</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
@@ -2113,32 +2113,32 @@
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Onbekend</t>
         </is>
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="M15" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="N15" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>Nee</t>
+          <t>Ja</t>
         </is>
       </c>
       <c r="P15" t="inlineStr">
@@ -2155,40 +2155,400 @@
         <v>20</v>
       </c>
       <c r="S15">
-        <v>128</v>
+        <v>160</v>
       </c>
       <c r="T15">
-        <v>38.3</v>
+        <v>34.3</v>
       </c>
       <c r="U15">
+        <v>6.5</v>
+      </c>
+      <c r="V15">
+        <v>6.5</v>
+      </c>
+      <c r="W15">
+        <v>6.1</v>
+      </c>
+      <c r="X15">
         <v>6.4</v>
       </c>
-      <c r="V15">
-        <v>6.4</v>
-      </c>
-      <c r="W15">
-        <v>5.9</v>
-      </c>
-      <c r="X15">
-        <v>6.3</v>
-      </c>
       <c r="Y15">
-        <v>7</v>
+        <v>7.2</v>
       </c>
       <c r="Z15">
         <v>6.2</v>
       </c>
       <c r="AA15">
+        <v>0</v>
+      </c>
+      <c r="AB15">
+        <v>0</v>
+      </c>
+      <c r="AC15">
+        <v>0</v>
+      </c>
+      <c r="AD15">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Vooropleiding</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="C16">
+        <v>2237</v>
+      </c>
+      <c r="D16">
+        <v>43</v>
+      </c>
+      <c r="E16">
+        <v>0.019</v>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Na CD</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>CD</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Onbekend</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="P16" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q16" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="R16">
+        <v>22</v>
+      </c>
+      <c r="S16">
+        <v>127</v>
+      </c>
+      <c r="T16">
+        <v>27.3</v>
+      </c>
+      <c r="U16">
+        <v>6.5</v>
+      </c>
+      <c r="V16">
+        <v>6.5</v>
+      </c>
+      <c r="W16">
+        <v>6.1</v>
+      </c>
+      <c r="X16">
+        <v>6.4</v>
+      </c>
+      <c r="Y16">
+        <v>7.2</v>
+      </c>
+      <c r="Z16">
+        <v>6.2</v>
+      </c>
+      <c r="AA16">
+        <v>0</v>
+      </c>
+      <c r="AB16">
+        <v>0</v>
+      </c>
+      <c r="AC16">
+        <v>0</v>
+      </c>
+      <c r="AD16">
+        <v>2022</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Vooropleiding</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>HO</t>
+        </is>
+      </c>
+      <c r="C17">
+        <v>2237</v>
+      </c>
+      <c r="D17">
+        <v>57</v>
+      </c>
+      <c r="E17">
+        <v>0.025</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Switch extern</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>HO</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="P17" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q17" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="R17">
+        <v>21</v>
+      </c>
+      <c r="S17">
+        <v>125</v>
+      </c>
+      <c r="T17">
+        <v>34.3</v>
+      </c>
+      <c r="U17">
+        <v>6.5</v>
+      </c>
+      <c r="V17">
+        <v>6.5</v>
+      </c>
+      <c r="W17">
+        <v>6.1</v>
+      </c>
+      <c r="X17">
+        <v>6.4</v>
+      </c>
+      <c r="Y17">
+        <v>7.2</v>
+      </c>
+      <c r="Z17">
+        <v>6.2</v>
+      </c>
+      <c r="AA17">
+        <v>0</v>
+      </c>
+      <c r="AB17">
+        <v>0</v>
+      </c>
+      <c r="AC17">
+        <v>0</v>
+      </c>
+      <c r="AD17">
+        <v>2020</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Vooropleiding</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Overig</t>
+        </is>
+      </c>
+      <c r="C18">
+        <v>2237</v>
+      </c>
+      <c r="D18">
+        <v>6</v>
+      </c>
+      <c r="E18">
+        <v>0.003</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Switch extern</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Overig</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>EM</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="P18" t="inlineStr">
+        <is>
+          <t>Ja</t>
+        </is>
+      </c>
+      <c r="Q18" t="inlineStr">
+        <is>
+          <t>Nee</t>
+        </is>
+      </c>
+      <c r="R18">
+        <v>20</v>
+      </c>
+      <c r="S18">
+        <v>130.5</v>
+      </c>
+      <c r="T18">
+        <v>31</v>
+      </c>
+      <c r="U18">
+        <v>6.5</v>
+      </c>
+      <c r="V18">
+        <v>6.5</v>
+      </c>
+      <c r="W18">
+        <v>6.1</v>
+      </c>
+      <c r="X18">
+        <v>6.4</v>
+      </c>
+      <c r="Y18">
+        <v>7.2</v>
+      </c>
+      <c r="Z18">
+        <v>6.2</v>
+      </c>
+      <c r="AA18">
+        <v>0.2</v>
+      </c>
+      <c r="AB18">
         <v>0.1</v>
       </c>
-      <c r="AB15">
-        <v>0.1</v>
-      </c>
-      <c r="AC15">
-        <v>0</v>
-      </c>
-      <c r="AD15">
-        <v>2015</v>
+      <c r="AC18">
+        <v>0</v>
+      </c>
+      <c r="AD18">
+        <v>2018</v>
       </c>
     </row>
   </sheetData>

</xml_diff>